<commit_message>
Strip stray footer legal bar from imported page body
The homepage import leaked the site's footer legal bar (DCGC logo, Disclaimer/
Privacy Policy/Code of Commitment/Responsible Disclosure links, copyright) and
the floating "Scroll To Top" widget into the page body. These live in
.copyright-wrap and #scrollToTopBtn, which sit OUTSIDE <footer> on the source,
so the existing footer removal missed them. Add both to the cleanup
transformer's removal list and rebundle so re-imports match the live page,
where this content belongs to the footer, not the body.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-home.report.xlsx
+++ b/tools/importer/reports/import-home.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["tabs-panel","hero-promo","hero-promo","hero-promo","carousel-banner","carousel-banner","columns-split","columns-split","columns-split","columns-split","columns-split","columns-split","columns-split","cards-product","cards-product","cards-product","cards-product","cards-product","cards-product","widget","cards-stats","cards-stats"]</t>
+    <t>["tabs-panel","hero-promo","hero-promo","hero-promo","carousel-banner","carousel-banner","carousel-banner","columns-split","columns-split","columns-split","columns-split","columns-split","columns-split","columns-split","cards-product","cards-product","cards-product","cards-product","cards-product","widget","cards-stats","cards-stats"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-09-09T15:24:08.457Z</t>
+    <t>2026-09-21T13:31:57.544Z</t>
   </si>
   <si>
     <t>Personal Banking | Internet Banking | Corporate, NRI Banking Services Online - Axis Bank</t>
@@ -73,7 +73,7 @@
     <t>accounts</t>
   </si>
   <si>
-    <t>2026-09-09T07:29:09.461Z</t>
+    <t>2026-09-09T15:24:53.332Z</t>
   </si>
   <si>
     <t>Savings Account - Open Bank Account Online in Minutes | Axis Bank</t>
@@ -91,7 +91,7 @@
     <t>cards/credit-card</t>
   </si>
   <si>
-    <t>2026-09-09T07:22:17.841Z</t>
+    <t>2026-09-09T15:25:05.275Z</t>
   </si>
   <si>
     <t>Credit Card - Apply for Credit Card Online &amp; Get Instant Approval | Axis Bank</t>

</xml_diff>